<commit_message>
FS-HU-21 a FS-HU-24 y FS-HU-05: Inicio con sesion, busqueda de profesionales con filtros y cercania, favoritos y resenas
Logo al Inicio, menu de la cuenta y diseno comun con menu lateral y barra inferior; portada redisenada; migraciones comuna/modalidad, favoritos y resenas; pruebas (backend 129, frontend 100) y documentacion (DAS v1.14, backlog, historias, Sprint 3, CP-036 a CP-049, defectos 8 a 14).
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I24"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="1.42578125" customWidth="1" style="5" min="1" max="1"/>
@@ -654,7 +654,7 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Planificada</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
@@ -668,7 +668,11 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>Implementada por Nicolás Silva y fusionada en main el 02-10-2026 (PR #8), sin Google Places ni mapa incorporado. 03-10-2026: el listado se amplió con la búsqueda avanzada (FS-HU-22) y cada ficha muestra calificación, comuna y modalidad. Falta la aceptación del Product Owner.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="9" t="inlineStr">
@@ -722,7 +726,7 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Planificada</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
@@ -736,7 +740,11 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr"/>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>03-10-2026: implementada junto con FS-HU-22 antes del inicio del Sprint 3. Con permiso de ubicación se filtra por distancia máxima (2, 5, 10 o 25 km) y se ordena por cercanía; sin permiso se informa y se puede buscar por comuna (escenario 2). La ubicación se redondea a unos 100 m y no se guarda ni se agrega a la dirección de la página (DAS, D23). Probada (CP-044 y CP-045); falta la DoD (revisión de código y PR). El mapa (FS-HU-06) sigue pendiente.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="9" t="inlineStr">
@@ -1280,7 +1288,159 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 23-09-2026 (épica E1). La portada la construyó Nicolás Silva (PR #2, 22-09-2026); el 23-09-2026 el Product Owner definió que es solo para quien no ha iniciado sesión: con la sesión iniciada se va directo al perfil y al cerrar sesión se vuelve a la portada. 23-09-2026: implementada y probada (CP-020 a CP-023); falta completar la DoD (revisión de código).</t>
+          <t>Agregada el 23-09-2026 (épica E1). La portada la construyó Nicolás Silva (PR #2, 22-09-2026); el 23-09-2026 el Product Owner definió que es solo para quien no ha iniciado sesión: con la sesión iniciada se va directo al perfil y al cerrar sesión se vuelve a la portada. 23-09-2026: implementada y probada (CP-020 a CP-023); falta completar la DoD (revisión de código). 03-10-2026: con la sesión iniciada la raíz lleva al Inicio (/inicio, FS-HU-21) en vez del perfil, y la portada se rediseñó con la propuesta "Tu salud y bienestar, en un solo lugar" y lo que ofrece FitSearch (CP-036 y CP-037).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>FS-HU-21</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Como un usuario, necesito un inicio con accesos a las secciones de la plataforma, mi objetivo, mi progreso y mis próximas citas, con la finalidad de orientarme y llegar rápido a lo que necesito.</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Inicio personalizado y navegación</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>Agregada el 03-10-2026 (épica E1) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Las secciones que aún no existen (centros de salud, gimnasios, farmacias, asistente IA, historial de chats y citas) se muestran como "Próximamente"; la barra de avance del objetivo esperará al gestor de alimentación (FS-HU-09 y FS-HU-10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>FS-HU-22</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Como un usuario, necesito buscar profesionales por texto y filtrarlos por especialidad, comuna, distancia, calificación y modalidad, con la finalidad de encontrar rápidamente al profesional que se ajusta a lo que busco.</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Búsqueda avanzada de profesionales</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>Agregada el 03-10-2026 (épica E3) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Incluye la búsqueda por cercanía de FS-HU-05 (distancia máxima y orden por cercanía). Requirió las columnas comuna y modalidad en profesionales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>FS-HU-23</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Como un usuario, necesito guardar profesionales como favoritos, con la finalidad de volver a encontrarlos fácilmente.</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Profesionales favoritos</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>Agregada el 03-10-2026 (épica E2) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Tabla favoritos (una fila por usuario y profesional).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>FS-HU-24</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Como un usuario, necesito calificar con estrellas a un profesional y comentar mi experiencia, con la finalidad de ayudar a otras personas a elegir y conocer la opinión de quienes ya se atendieron.</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Calificar y reseñar profesionales</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>En Proceso</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>Agregada el 03-10-2026 (épica E2) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Tabla resenas (una por usuario y profesional). Solo las cuentas de usuario califican; cuando exista FS-HU-14 se restringirá a quienes tuvieron una reserva confirmada.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revision de codigo aprobada (PR #9 y #10) y aceptacion del PO de las historias del Sprint 2
FS-HU-02 y FS-HU-15 a FS-HU-20 aceptadas. Revision de 2 h de Luis registrada en el Sprint Backlog del Sprint 2. Matriz de control de cambio, EDT y analisis de ingresos, Guia 2.4, control y README actualizados.
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="B1:I28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="1.42578125" customWidth="1" style="5" min="1" max="1"/>
@@ -632,7 +632,7 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>Se agregó el sexo a los datos básicos (Sprint 1) para estimar el requerimiento calórico con la ecuación de Mifflin-St Jeor. Sprint 1: aceptada por el Product Owner el 24-09-2026 (CP-001 a CP-007 aprobados). Excepción a DoD-03 (sin pull request en el Sprint 1) y revisión de código posterior aprobada por Luis Méndez en el PR #6 (24-09-2026). 24-09-2026: por decisión del Product Owner se agregó al asistente un primer paso para elegir el tipo de cuenta (usuario o profesional), que antes se elegía en el registro; el asistente queda de 5 pasos. Implementado y probado (CP-027 y CP-028); pendiente la aceptación del Product Owner del criterio nuevo.</t>
+          <t>Se agregó el sexo a los datos básicos (Sprint 1) para estimar el requerimiento calórico con la ecuación de Mifflin-St Jeor. Sprint 1: aceptada por el Product Owner el 24-09-2026 (CP-001 a CP-007 aprobados). Excepción a DoD-03 (sin pull request en el Sprint 1) y revisión de código posterior aprobada por Luis Méndez en el PR #6 (24-09-2026). 24-09-2026: por decisión del Product Owner se agregó al asistente un primer paso para elegir el tipo de cuenta (usuario o profesional), que antes se elegía en el registro; el asistente queda de 5 pasos. Implementado y probado (CP-027 y CP-028); pendiente la aceptación del Product Owner del criterio nuevo. 03-10-2026: el Product Owner aceptó el criterio nuevo del tipo de cuenta, con la revisión de código aprobada por Luis Méndez en el PR #9 (con la misma excepción a DoD-03).</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>03-10-2026: implementada junto con FS-HU-22 antes del inicio del Sprint 3. Con permiso de ubicación se filtra por distancia máxima (2, 5, 10 o 25 km) y se ordena por cercanía; sin permiso se informa y se puede buscar por comuna (escenario 2). La ubicación se redondea a unos 100 m y no se guarda ni se agrega a la dirección de la página (DAS, D23). Probada (CP-044 y CP-045); falta la DoD (revisión de código y PR). El mapa (FS-HU-06) sigue pendiente.</t>
+          <t>03-10-2026: implementada junto con FS-HU-22 antes del inicio del Sprint 3. Con permiso de ubicación se filtra por distancia máxima (2, 5, 10 o 25 km) y se ordena por cercanía; sin permiso se informa y se puede buscar por comuna (escenario 2). La ubicación se redondea a unos 100 m y no se guarda ni se agrega a la dirección de la página (DAS, D23). Probada (CP-044 y CP-045); falta la DoD (revisión de código y PR). El mapa (FS-HU-06) sigue pendiente. 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F19" s="9" t="n">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 21-09-2026 (épica E1) por decisión del Product Owner, a partir del diseño de las pantallas de acceso. El enlace vence a los 60 minutos y sirve una sola vez. 21-09-2026: implementada y probada (CP-011 a CP-013); falta configurar la cuenta de correo SMTP para el envío real y completar la DoD (revisión de código y PR).</t>
+          <t>Agregada el 21-09-2026 (épica E1) por decisión del Product Owner, a partir del diseño de las pantallas de acceso. El enlace vence a los 60 minutos y sirve una sola vez. 21-09-2026: implementada y probada (CP-011 a CP-013); falta configurar la cuenta de correo SMTP para el envío real y completar la DoD (revisión de código y PR). 03-10-2026: aceptada por el Product Owner, con la revisión de código aprobada por Luis Méndez en el PR #9. Observación: falta configurar la cuenta SMTP para el envío real; mientras tanto el enlace se muestra en la consola del backend. Excepción a DoD-03: el código llegó a main sin pull request y se revisó después en el PR #9.</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F20" s="9" t="n">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 21-09-2026 (épica E1). Solo Google; el acceso con Apple quedó fuera por decisión del Product Owner. 24-09-2026: creada la cuenta fitsearchoficial@gmail.com y el ID de cliente OAuth en Google Cloud; implementada con el botón oficial de Google Identity Services y la verificación del token en el backend (POST /api/auth/google). La aplicación queda en modo de prueba en Google Cloud, con los correos del equipo como usuarios de prueba. Pendiente: ejecutar los casos de prueba manuales CP-024 y CP-025 con la cuenta de Google y completar la DoD (revisión de código y PR). 24-09-2026: entrar con Google ya no define el rol de la cuenta (se creaba con el rol que estuviera marcado en el registro, lo que provocaba equivocaciones); el tipo de cuenta se elige en el perfil.</t>
+          <t>Agregada el 21-09-2026 (épica E1). Solo Google; el acceso con Apple quedó fuera por decisión del Product Owner. 24-09-2026: creada la cuenta fitsearchoficial@gmail.com y el ID de cliente OAuth en Google Cloud; implementada con el botón oficial de Google Identity Services y la verificación del token en el backend (POST /api/auth/google). La aplicación queda en modo de prueba en Google Cloud, con los correos del equipo como usuarios de prueba. Pendiente: ejecutar los casos de prueba manuales CP-024 y CP-025 con la cuenta de Google y completar la DoD (revisión de código y PR). 24-09-2026: entrar con Google ya no define el rol de la cuenta (se creaba con el rol que estuviera marcado en el registro, lo que provocaba equivocaciones); el tipo de cuenta se elige en el perfil. 03-10-2026: aceptada por el Product Owner, con la revisión de código aprobada por Luis Méndez en el PR #9. Observación: faltan los casos manuales CP-024 y CP-025, que requieren iniciar sesión con una cuenta de Google del equipo. Excepción a DoD-03: el código llegó a main sin pull request y se revisó después en el PR #9.</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F21" s="9" t="n">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 21-09-2026 (épica E1) junto con la nueva identidad visual de las pantallas de acceso (logo, paleta azul y naranja). El registro no incluye la casilla de términos y condiciones. 21-09-2026: implementada y probada (CP-008 a CP-010); falta completar la DoD (revisión de código y PR). 24-09-2026: se quitó del registro la elección del rol (pasó al asistente de perfil, FS-HU-02); toda cuenta nueva se crea como usuario. CP-008 se rehizo con el flujo nuevo.</t>
+          <t>Agregada el 21-09-2026 (épica E1) junto con la nueva identidad visual de las pantallas de acceso (logo, paleta azul y naranja). El registro no incluye la casilla de términos y condiciones. 21-09-2026: implementada y probada (CP-008 a CP-010); falta completar la DoD (revisión de código y PR). 24-09-2026: se quitó del registro la elección del rol (pasó al asistente de perfil, FS-HU-02); toda cuenta nueva se crea como usuario. CP-008 se rehizo con el flujo nuevo. 03-10-2026: aceptada por el Product Owner, con la revisión de código aprobada por Luis Méndez en el PR #9. Excepción a DoD-03: el código llegó a main sin pull request y se revisó después en el PR #9.</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F22" s="9" t="n">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 21-09-2026 (épica E1) junto con el asistente de perfil de 5 pasos y el resumen con "Editar" (rediseño de FS-HU-02). 21-09-2026: implementada y probada (CP-018); falta completar la DoD (revisión de código y PR).</t>
+          <t>Agregada el 21-09-2026 (épica E1) junto con el asistente de perfil de 5 pasos y el resumen con "Editar" (rediseño de FS-HU-02). 21-09-2026: implementada y probada (CP-018); falta completar la DoD (revisión de código y PR). 03-10-2026: aceptada por el Product Owner, con la revisión de código aprobada por Luis Méndez en el PR #9. Excepción a DoD-03: el código llegó a main sin pull request y se revisó después en el PR #9.</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F23" s="9" t="n">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 21-09-2026 (épica E1). Dato sensible: solo opciones de catálogo, sin texto libre, y solo su dueño lo consulta (DAS, QS7). 21-09-2026: implementada y probada (CP-014 a CP-017); falta completar la DoD (revisión de código y PR).</t>
+          <t>Agregada el 21-09-2026 (épica E1). Dato sensible: solo opciones de catálogo, sin texto libre, y solo su dueño lo consulta (DAS, QS7). 21-09-2026: implementada y probada (CP-014 a CP-017); falta completar la DoD (revisión de código y PR). 03-10-2026: aceptada por el Product Owner, con la revisión de código aprobada por Luis Méndez en el PR #9. Excepción a DoD-03: el código llegó a main sin pull request y se revisó después en el PR #9.</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F24" s="9" t="n">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 23-09-2026 (épica E1). La portada la construyó Nicolás Silva (PR #2, 22-09-2026); el 23-09-2026 el Product Owner definió que es solo para quien no ha iniciado sesión: con la sesión iniciada se va directo al perfil y al cerrar sesión se vuelve a la portada. 23-09-2026: implementada y probada (CP-020 a CP-023); falta completar la DoD (revisión de código). 03-10-2026: con la sesión iniciada la raíz lleva al Inicio (/inicio, FS-HU-21) en vez del perfil, y la portada se rediseñó con la propuesta "Tu salud y bienestar, en un solo lugar" y lo que ofrece FitSearch (CP-036 y CP-037).</t>
+          <t>Agregada el 23-09-2026 (épica E1). La portada la construyó Nicolás Silva (PR #2, 22-09-2026); el 23-09-2026 el Product Owner definió que es solo para quien no ha iniciado sesión: con la sesión iniciada se va directo al perfil y al cerrar sesión se vuelve a la portada. 23-09-2026: implementada y probada (CP-020 a CP-023); falta completar la DoD (revisión de código). 03-10-2026: con la sesión iniciada la raíz lleva al Inicio (/inicio, FS-HU-21) en vez del perfil, y la portada se rediseñó con la propuesta "Tu salud y bienestar, en un solo lugar" y lo que ofrece FitSearch (CP-036 y CP-037). 03-10-2026: aceptada por el Product Owner, con la revisión de código aprobada por Luis Méndez en el PR #9. El código de la portada entró por el PR #2, que se fusionó sin revisión; la revisión se hizo después en el PR #9.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 03-10-2026 (épica E1) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Las secciones que aún no existen (centros de salud, gimnasios, farmacias, asistente IA, historial de chats y citas) se muestran como "Próximamente"; la barra de avance del objetivo esperará al gestor de alimentación (FS-HU-09 y FS-HU-10).</t>
+          <t>Agregada el 03-10-2026 (épica E1) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Las secciones que aún no existen (centros de salud, gimnasios, farmacias, asistente IA, historial de chats y citas) se muestran como "Próximamente"; la barra de avance del objetivo esperará al gestor de alimentación (FS-HU-09 y FS-HU-10). 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 03-10-2026 (épica E3) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Incluye la búsqueda por cercanía de FS-HU-05 (distancia máxima y orden por cercanía). Requirió las columnas comuna y modalidad en profesionales.</t>
+          <t>Agregada el 03-10-2026 (épica E3) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Incluye la búsqueda por cercanía de FS-HU-05 (distancia máxima y orden por cercanía). Requirió las columnas comuna y modalidad en profesionales. 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 03-10-2026 (épica E2) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Tabla favoritos (una fila por usuario y profesional).</t>
+          <t>Agregada el 03-10-2026 (épica E2) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Tabla favoritos (una fila por usuario y profesional). 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 03-10-2026 (épica E2) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Tabla resenas (una por usuario y profesional). Solo las cuentas de usuario califican; cuando exista FS-HU-14 se restringirá a quienes tuvieron una reserva confirmada.</t>
+          <t>Agregada el 03-10-2026 (épica E2) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Tabla resenas (una por usuario y profesional). Solo las cuentas de usuario califican; cuando exista FS-HU-14 se restringirá a quienes tuvieron una reserva confirmada. 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FS-HU-03 aceptada por el PO (PR #8 revisado)
Product Backlog, Sprint Backlog del Sprint 2, Guia 2.4 y control actualizados.
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -654,7 +654,7 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F7" s="9" t="n">
@@ -670,7 +670,7 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Implementada por Nicolás Silva y fusionada en main el 02-10-2026 (PR #8), sin Google Places ni mapa incorporado. 03-10-2026: el listado se amplió con la búsqueda avanzada (FS-HU-22) y cada ficha muestra calificación, comuna y modalidad. Falta la aceptación del Product Owner.</t>
+          <t>Implementada por Nicolás Silva y fusionada en main el 02-10-2026 (PR #8), sin Google Places ni mapa incorporado. 03-10-2026: el listado se amplió con la búsqueda avanzada (FS-HU-22) y cada ficha muestra calificación, comuna y modalidad. 03-10-2026: aceptada por el Product Owner; el PR #8 cumple DoD-03 y DoD-04 (revisión aprobada por Rodrigo Cárcamo Rojas). La ampliación con la búsqueda avanzada se sigue en FS-HU-22.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Concilia backlogs y corrige sesiones y navegación por rol
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -674,7 +674,7 @@
         </ns0:is>
       </ns0:c>
     </ns0:row>
-    <ns0:row r="8">
+    <ns0:row r="8" ht="120" customHeight="1">
       <ns0:c r="B8" s="9" t="inlineStr">
         <ns0:is>
           <ns0:t>FS-HU-04</ns0:t>
@@ -690,10 +690,8 @@
           <ns0:t>Perfil de profesional</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="E8" s="9" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Planificada</ns0:t>
-        </ns0:is>
+      <ns0:c r="E8" s="9" t="str">
+        <ns0:v>En Proceso</ns0:v>
       </ns0:c>
       <ns0:c r="F8" s="9" t="n">
         <ns0:v>5</ns0:v>
@@ -706,7 +704,9 @@
           <ns0:t>Alta</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="I8" s="9" t="inlineStr"/>
+      <ns0:c r="I8" s="9" t="str">
+        <ns0:v>Implementado por Luis (PR #12), con ajustes de Rodri (#13). Pendiente de aceptación del PO. Actualizado 10-10-2026.</ns0:v>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="9">
       <ns0:c r="B9" s="9" t="inlineStr">
@@ -986,7 +986,7 @@
         <ns0:v>Agregada 14-09-2026, E2/CU-07. Avance técnico 10-10-2026: API e insignias probadas, en revisión. Pantalla y cuentas administrativas pendientes de alcance del PO. Sprint 5 si hay capacidad; sin aceptación. Trello: https://trello.com/c/4CaN8UAs</ns0:v>
       </ns0:c>
     </ns0:row>
-    <ns0:row r="17">
+    <ns0:row r="17" ht="340" customHeight="1">
       <ns0:c r="B17" s="9" t="inlineStr">
         <ns0:is>
           <ns0:t>FS-HU-13</ns0:t>
@@ -1011,17 +1011,15 @@
         <ns0:v>5</ns0:v>
       </ns0:c>
       <ns0:c r="G17" s="9" t="n">
-        <ns0:v>2</ns0:v>
+        <ns0:v>3</ns0:v>
       </ns0:c>
       <ns0:c r="H17" s="9" t="inlineStr">
         <ns0:is>
           <ns0:t>Alta</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="I17" s="9" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Agregada el 15-09-2026 (épica E7 Reservas) por decisión del Product Owner y el equipo. Reserva básica sin pagos ni calendarios externos.</ns0:t>
-        </ns0:is>
+      <ns0:c r="I17" s="9" t="str">
+        <ns0:v>Agregada el 15-09-2026 (épica E7 Reservas) por decisión del Product Owner y el equipo. Reserva básica sin pagos ni calendarios externos. Replanificada a Sprint 3 (Trello). Sin iniciar; sin responsable ni estimación.</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="18">

</xml_diff>

<commit_message>
Corrige superposición de horas, retiro de horarios y notas del backlog
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias de Usuario" sheetId="1" r:id="R7c8b7521e6844ba5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructivo" sheetId="2" r:id="R5c89d4e3d1294b56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias de Usuario" sheetId="1" r:id="Rb6fdbfbf9e1b48e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructivo" sheetId="2" r:id="Re364c67580fb49aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -472,7 +472,7 @@
     <x:col min="6" max="6" width="11.85546875" style="5" customWidth="1"/>
     <x:col min="7" max="7" width="16.140625" style="5" customWidth="1"/>
     <x:col min="8" max="8" width="17.85546875" style="5" customWidth="1"/>
-    <x:col min="9" max="9" width="12.28515625" style="5" customWidth="1"/>
+    <x:col min="9" max="9" width="36" style="5" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="2.140625" style="5" customWidth="1"/>
     <x:col min="11" max="16384" width="11.42578125" style="5" customWidth="1"/>
   </x:cols>
@@ -979,7 +979,7 @@
         <x:v>Agregada 14-09-2026, E2/CU-07. Avance técnico 10-10-2026: API e insignias probadas, en revisión. Pantalla y cuentas administrativas pendientes de alcance del PO. Sprint 5 si hay capacidad; sin aceptación. Trello: https://trello.com/c/4CaN8UAs</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="220" customHeight="1">
+    <x:row r="17" ht="300" customHeight="1">
       <x:c r="B17" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">FS-HU-13</x:t>
@@ -1010,10 +1010,11 @@
         </x:is>
       </x:c>
       <x:c r="I17" s="9" t="str">
-        <x:v>Arrastre a Sprint 3. Luis implementó API y pantalla; valida futuros, superposición y propiedad. MySQL real aprobado. En revisión, pendiente de fusión y aceptación. 11-10-2026.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="220" customHeight="1">
+        <x:v>Agregada el 15-09-2026 (épica E7 Reservas) por decisión del Product Owner y el equipo. Reserva básica sin pagos ni calendarios externos. Replanificada a Sprint 3 (Trello). Sin iniciar; sin responsable ni estimación.
+Avance al 12-10-2026: Arrastre a Sprint 3. Luis implementó API y pantalla; valida futuros, superposición y propiedad. MySQL real aprobado. En revisión, pendiente de fusión y aceptación. 11-10-2026. Corrección del PR #21: comparación en segundos, retiro sin perder historial y prueba MySQL reproducible. En revisión.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="300" customHeight="1">
       <x:c r="B18" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">FS-HU-14</x:t>
@@ -1044,7 +1045,8 @@
         </x:is>
       </x:c>
       <x:c r="I18" s="9" t="str">
-        <x:v>Luis implementó reserva con mensaje obligatorio, transacción para una activa por bloque, confirmación, cancelación e historial. MySQL real aprobado. En revisión, pendiente de fusión y aceptación. 11-10-2026.</x:v>
+        <x:v>Agregada el 15-09-2026 (épica E7 Reservas). Al presionar "Reservar" el usuario escribe un mensaje breve obligatorio para el profesional.
+Avance al 12-10-2026: Luis implementó reserva con mensaje obligatorio, transacción para una activa por bloque, confirmación, cancelación e historial. MySQL real aprobado. En revisión, pendiente de fusión y aceptación. 11-10-2026. Corrección del PR #21: comparación en segundos, retiro sin perder historial y prueba MySQL reproducible. En revisión.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">

</xml_diff>

<commit_message>
Registra decisiones del PO, casos CP-069 a CP-078 y defectos 25 y 26
FS-HU-04 aceptada por el PO; FS-HU-12 en proceso en el Sprint 3. Planilla con 78 casos (75 aprobados) y celdas de CP-061 a CP-068 ordenadas. Registro de Defectos con los defectos 25 (corregido) y 26 (abierto, PR #22). Guía 2.4 y control actualizados al 12-10-2026.
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -670,7 +670,7 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F8" s="9" t="n">
@@ -687,7 +687,8 @@
       <c r="I8" s="9" t="inlineStr">
         <is>
           <t>06-10-2026 (cierre del Sprint 2): implementada por Luis Méndez en el PR #11 (03-10-2026), en corrección antes de fusionar; pasa al Sprint 3.
-Implementado por Luis (PR #12), con ajustes de Rodri (#13). Pendiente de aceptación del PO. Actualizado 10-10-2026.</t>
+Implementado por Luis (PR #12), con ajustes de Rodri (#13). Pendiente de aceptación del PO. Actualizado 10-10-2026.
+12-10-2026: aceptada por el Product Owner (Rodrigo Cárcamo Rojas).</t>
         </is>
       </c>
     </row>
@@ -955,14 +956,16 @@
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Planificada</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="F16" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="9" t="n">
-        <v>5</v>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
@@ -971,7 +974,8 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>Agregada 14-09-2026, E2/CU-07. Avance técnico 10-10-2026: API e insignias probadas, en revisión. Pantalla y cuentas administrativas pendientes de alcance del PO. Sprint 5 si hay capacidad; sin aceptación. Trello: https://trello.com/c/4CaN8UAs</t>
+          <t>Agregada 14-09-2026, E2/CU-07. Avance técnico 10-10-2026: API e insignias probadas, en revisión. Pantalla y cuentas administrativas pendientes de alcance del PO. Sprint 5 si hay capacidad; sin aceptación. Trello: https://trello.com/c/4CaN8UAs
+12-10-2026: implementada por Luis Méndez durante el Sprint 3 (PR #15, #19 y #20, fusionados entre el 10 y el 11-10-2026). El Product Owner la reubica en el Sprint 3. Pendiente de aceptación del PO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza estados tras fusionar el PR #22: README, DAS 1.22, backlogs y documentos del Sprint 3
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -764,7 +764,8 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>Mapa/lista integrado por Luis; conserva filtros y página. Pruebas locales aprobadas. Falta clave y validación real Google Maps; revisión y aceptación pendientes. 11-10-2026.</t>
+          <t>Mapa/lista integrado por Luis; conserva filtros y página. Pruebas locales aprobadas. Falta clave y validación real Google Maps; revisión y aceptación pendientes. 11-10-2026.
+12-10-2026: los PR #21 y #22 se fusionaron en main (merge 662e79c). Google Maps real comprobado con una Demo Key, sin facturación: marcadores, filtros, Lista/Mapa y paginación. Falta ejecutar CP-078 sobre main y la aceptación del PO.</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1015,8 @@
       <c r="I17" s="9" t="inlineStr">
         <is>
           <t>Agregada el 15-09-2026 (épica E7 Reservas) por decisión del Product Owner y el equipo. Reserva básica sin pagos ni calendarios externos. Replanificada a Sprint 3 (Trello). Sin iniciar; sin responsable ni estimación.
-Avance al 12-10-2026: Arrastre a Sprint 3. Luis implementó API y pantalla; valida futuros, superposición y propiedad. MySQL real aprobado. En revisión, pendiente de fusión y aceptación. 11-10-2026. Corrección del PR #21: comparación en segundos, retiro sin perder historial y prueba MySQL reproducible. En revisión.</t>
+Avance al 12-10-2026: Arrastre a Sprint 3. Luis implementó API y pantalla; valida futuros, superposición y propiedad. MySQL real aprobado. En revisión, pendiente de fusión y aceptación. 11-10-2026. Corrección del PR #21: comparación en segundos, retiro sin perder historial y prueba MySQL reproducible. En revisión.
+12-10-2026: los PR #21 y #22 se fusionaron en main (merge 662e79c); 55/55 comprobaciones con MySQL real sobre main. Pendiente de aceptación del PO.</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1094,8 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 21-09-2026 (épica E1) por decisión del Product Owner, a partir del diseño de las pantallas de acceso. El enlace vence a los 60 minutos y sirve una sola vez. 21-09-2026: implementada y probada (CP-011 a CP-013); falta configurar la cuenta de correo SMTP para el envío real y completar la DoD (revisión de código y PR). 03-10-2026: aceptada por el Product Owner, con la revisión de código aprobada por Luis Méndez en el PR #9. Observación: falta configurar la cuenta SMTP para el envío real; mientras tanto el enlace se muestra en la consola del backend. Excepción a DoD-03: el código llegó a main sin pull request y se revisó después en el PR #9.</t>
+          <t>Agregada el 21-09-2026 (épica E1) por decisión del Product Owner, a partir del diseño de las pantallas de acceso. El enlace vence a los 60 minutos y sirve una sola vez. 21-09-2026: implementada y probada (CP-011 a CP-013); falta configurar la cuenta de correo SMTP para el envío real y completar la DoD (revisión de código y PR). 03-10-2026: aceptada por el Product Owner, con la revisión de código aprobada por Luis Méndez en el PR #9. Observación: falta configurar la cuenta SMTP para el envío real; mientras tanto el enlace se muestra en la consola del backend. Excepción a DoD-03: el código llegó a main sin pull request y se revisó después en el PR #9.
+12-10-2026: Luis Méndez comprobó el envío real por SMTP (Gmail): el correo de recuperación llegó a la bandeja de entrada y la recuperación se completó (Proveedores_Reales_2026-10-12.json, en Plan de Pruebas). Las credenciales quedan solo en el .env local.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aceptacion del PO de 8 historias del Sprint 3 y horas del Sprint 3 con tope de 5 h diarias
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -477,7 +477,7 @@
     <col width="11.85546875" customWidth="1" style="5" min="6" max="6"/>
     <col width="16.140625" customWidth="1" style="5" min="7" max="7"/>
     <col width="17.85546875" customWidth="1" style="5" min="8" max="8"/>
-    <col width="36" customWidth="1" style="5" min="9" max="9"/>
+    <col width="70" customWidth="1" style="5" min="9" max="9"/>
     <col width="2.140625" customWidth="1" style="5" min="10" max="10"/>
     <col width="11.42578125" customWidth="1" style="5" min="11" max="16384"/>
   </cols>
@@ -538,7 +538,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="70" customHeight="1">
       <c r="B5" s="9" t="inlineStr">
         <is>
           <t>FS-HU-01</t>
@@ -576,7 +576,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="205" customHeight="1">
       <c r="B6" s="9" t="inlineStr">
         <is>
           <t>FS-HU-02</t>
@@ -614,7 +614,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="115" customHeight="1">
       <c r="B7" s="9" t="inlineStr">
         <is>
           <t>FS-HU-03</t>
@@ -652,7 +652,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="120" customHeight="1">
+    <row r="8" ht="130" customHeight="1">
       <c r="B8" s="9" t="inlineStr">
         <is>
           <t>FS-HU-04</t>
@@ -692,7 +692,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="190" customHeight="1">
       <c r="B9" s="9" t="inlineStr">
         <is>
           <t>FS-HU-05</t>
@@ -710,7 +710,7 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F9" s="9" t="n">
@@ -726,11 +726,12 @@
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>03-10-2026: implementada junto con FS-HU-22 antes del inicio del Sprint 3. Con permiso de ubicación se filtra por distancia máxima (2, 5, 10 o 25 km) y se ordena por cercanía; sin permiso se informa y se puede buscar por comuna (escenario 2). La ubicación se redondea a unos 100 m y no se guarda ni se agrega a la dirección de la página (DAS, D23). Probada (CP-044 y CP-045); falta la DoD (revisión de código y PR). El mapa (FS-HU-06) sigue pendiente. 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="220" customHeight="1">
+          <t>03-10-2026: implementada junto con FS-HU-22 antes del inicio del Sprint 3. Con permiso de ubicación se filtra por distancia máxima (2, 5, 10 o 25 km) y se ordena por cercanía; sin permiso se informa y se puede buscar por comuna (escenario 2). La ubicación se redondea a unos 100 m y no se guarda ni se agrega a la dirección de la página (DAS, D23). Probada (CP-044 y CP-045); falta la DoD (revisión de código y PR). El mapa (FS-HU-06) sigue pendiente. 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.
+12-10-2026: aceptada por el Product Owner. Casos CP-044 y CP-045 aprobados; revisión de código de Luis Méndez en el PR #10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="130" customHeight="1">
       <c r="B10" s="9" t="inlineStr">
         <is>
           <t>FS-HU-06</t>
@@ -939,7 +940,7 @@
       </c>
       <c r="I15" s="9" t="inlineStr"/>
     </row>
-    <row r="16" ht="300" customHeight="1">
+    <row r="16" ht="220" customHeight="1">
       <c r="B16" s="9" t="inlineStr">
         <is>
           <t>FS-HU-12</t>
@@ -957,7 +958,7 @@
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F16" s="9" t="n">
@@ -976,11 +977,12 @@
       <c r="I16" s="9" t="inlineStr">
         <is>
           <t>Agregada 14-09-2026, E2/CU-07. Avance técnico 10-10-2026: API e insignias probadas, en revisión. Pantalla y cuentas administrativas pendientes de alcance del PO. Sprint 5 si hay capacidad; sin aceptación. Trello: https://trello.com/c/4CaN8UAs
-12-10-2026: implementada por Luis Méndez durante el Sprint 3 (PR #15, #19 y #20, fusionados entre el 10 y el 11-10-2026). El Product Owner la reubica en el Sprint 3. Pendiente de aceptación del PO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="300" customHeight="1">
+12-10-2026: implementada por Luis Méndez durante el Sprint 3 (PR #15, #19 y #20, fusionados entre el 10 y el 11-10-2026). El Product Owner la reubica en el Sprint 3. Pendiente de aceptación del PO.
+12-10-2026: aceptada por el Product Owner, con observación. Casos CP-061 a CP-068 aprobados; revisión de código de Rodrigo Cárcamo Rojas en los PR #15, #19 y #20. Observación: al cambiar de especialidad se reinicia el cupo de cargas de documentos (pendiente menor).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="280" customHeight="1">
       <c r="B17" s="9" t="inlineStr">
         <is>
           <t>FS-HU-13</t>
@@ -998,7 +1000,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F17" s="9" t="n">
@@ -1016,11 +1018,12 @@
         <is>
           <t>Agregada el 15-09-2026 (épica E7 Reservas) por decisión del Product Owner y el equipo. Reserva básica sin pagos ni calendarios externos. Replanificada a Sprint 3 (Trello). Sin iniciar; sin responsable ni estimación.
 Avance al 12-10-2026: Arrastre a Sprint 3. Luis implementó API y pantalla; valida futuros, superposición y propiedad. MySQL real aprobado. En revisión, pendiente de fusión y aceptación. 11-10-2026. Corrección del PR #21: comparación en segundos, retiro sin perder historial y prueba MySQL reproducible. En revisión.
-12-10-2026: los PR #21 y #22 se fusionaron en main (merge 662e79c); 55/55 comprobaciones con MySQL real sobre main. Pendiente de aceptación del PO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="300" customHeight="1">
+12-10-2026: los PR #21 y #22 se fusionaron en main (merge 662e79c); 55/55 comprobaciones con MySQL real sobre main. Pendiente de aceptación del PO.
+12-10-2026: aceptada por el Product Owner. Casos CP-069 a CP-071 aprobados contra MySQL real; revisión de código de Rodrigo Cárcamo Rojas en los PR #21 y #22.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="340" customHeight="1">
       <c r="B18" s="9" t="inlineStr">
         <is>
           <t>FS-HU-14</t>
@@ -1038,7 +1041,7 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F18" s="9" t="n">
@@ -1056,11 +1059,12 @@
         <is>
           <t>Agregada el 15-09-2026 (épica E7 Reservas). Al presionar "Reservar" el usuario escribe un mensaje breve obligatorio para el profesional.
 Avance al 12-10-2026: Luis implementó reserva con mensaje obligatorio, transacción para una activa por bloque, confirmación, cancelación e historial. MySQL real aprobado. En revisión, pendiente de fusión y aceptación. 11-10-2026. Corrección del PR #21: comparación en segundos, retiro sin perder historial y prueba MySQL reproducible. En revisión.
-12-10-2026: el Product Owner definió como máximo una reserva activa (pendiente o confirmada) por usuario con cada profesional; las citas que ya pasaron no cuentan. Implementado en el PR #22 (Luis Méndez, con la corrección de Rodrigo Cárcamo del defecto 26), fusionado el 12-10-2026. Pendiente de aceptación del PO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
+12-10-2026: el Product Owner definió como máximo una reserva activa (pendiente o confirmada) por usuario con cada profesional; las citas que ya pasaron no cuentan. Implementado en el PR #22 (Luis Méndez, con la corrección de Rodrigo Cárcamo del defecto 26), fusionado el 12-10-2026. Pendiente de aceptación del PO.
+12-10-2026: aceptada por el Product Owner, con observación. Casos CP-072 a CP-075, CP-079 y CP-080 aprobados; revisión de código de Rodrigo Cárcamo Rojas en los PR #21 y #22. Observación: la corrección del defecto 26 (commit 4728310, de Rodrigo Cárcamo Rojas) queda pendiente de revisión por otro integrante (DoD-04).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="235" customHeight="1">
       <c r="B19" s="9" t="inlineStr">
         <is>
           <t>FS-HU-15</t>
@@ -1099,7 +1103,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="265" customHeight="1">
       <c r="B20" s="9" t="inlineStr">
         <is>
           <t>FS-HU-16</t>
@@ -1137,7 +1141,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="175" customHeight="1">
       <c r="B21" s="9" t="inlineStr">
         <is>
           <t>FS-HU-17</t>
@@ -1175,7 +1179,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="115" customHeight="1">
       <c r="B22" s="9" t="inlineStr">
         <is>
           <t>FS-HU-18</t>
@@ -1213,7 +1217,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="115" customHeight="1">
       <c r="B23" s="9" t="inlineStr">
         <is>
           <t>FS-HU-19</t>
@@ -1251,7 +1255,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="205" customHeight="1">
       <c r="B24" s="9" t="inlineStr">
         <is>
           <t>FS-HU-20</t>
@@ -1289,7 +1293,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="250" customHeight="1">
       <c r="B25" s="9" t="inlineStr">
         <is>
           <t>FS-HU-21</t>
@@ -1307,7 +1311,7 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F25" s="9" t="n">
@@ -1323,11 +1327,12 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 03-10-2026 (épica E1) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Las secciones que aún no existen (centros de salud, gimnasios, farmacias, asistente IA, historial de chats y citas) se muestran como "Próximamente"; la barra de avance del objetivo esperará al gestor de alimentación (FS-HU-09 y FS-HU-10). 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
+          <t>Agregada el 03-10-2026 (épica E1) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Las secciones que aún no existen (centros de salud, gimnasios, farmacias, asistente IA, historial de chats y citas) se muestran como "Próximamente"; la barra de avance del objetivo esperará al gestor de alimentación (FS-HU-09 y FS-HU-10). 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.
+12-10-2026: aceptada por el Product Owner. Casos CP-037 a CP-041 y CP-049 aprobados; revisión de código de Luis Méndez en el PR #10. Los cambios del menú del PR #13 los revisó Luis Méndez al integrarlos en el PR #15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="205" customHeight="1">
       <c r="B26" s="9" t="inlineStr">
         <is>
           <t>FS-HU-22</t>
@@ -1345,7 +1350,7 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F26" s="9" t="n">
@@ -1361,11 +1366,12 @@
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 03-10-2026 (épica E3) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Incluye la búsqueda por cercanía de FS-HU-05 (distancia máxima y orden por cercanía). Requirió las columnas comuna y modalidad en profesionales. 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
+          <t>Agregada el 03-10-2026 (épica E3) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Incluye la búsqueda por cercanía de FS-HU-05 (distancia máxima y orden por cercanía). Requirió las columnas comuna y modalidad en profesionales. 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.
+12-10-2026: aceptada por el Product Owner. Casos CP-042 y CP-043 aprobados; revisión de código de Luis Méndez en el PR #10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="175" customHeight="1">
       <c r="B27" s="9" t="inlineStr">
         <is>
           <t>FS-HU-23</t>
@@ -1383,7 +1389,7 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F27" s="9" t="n">
@@ -1399,11 +1405,12 @@
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 03-10-2026 (épica E2) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Tabla favoritos (una fila por usuario y profesional). 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
+          <t>Agregada el 03-10-2026 (épica E2) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Tabla favoritos (una fila por usuario y profesional). 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.
+12-10-2026: aceptada por el Product Owner. Caso CP-046 aprobado; revisión de código de Luis Méndez en el PR #10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="205" customHeight="1">
       <c r="B28" s="9" t="inlineStr">
         <is>
           <t>FS-HU-24</t>
@@ -1421,7 +1428,7 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F28" s="9" t="n">
@@ -1437,7 +1444,8 @@
       </c>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 03-10-2026 (épica E2) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Tabla resenas (una por usuario y profesional). Solo las cuentas de usuario califican; cuando exista FS-HU-14 se restringirá a quienes tuvieron una reserva confirmada. 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.</t>
+          <t>Agregada el 03-10-2026 (épica E2) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Tabla resenas (una por usuario y profesional). Solo las cuentas de usuario califican; cuando exista FS-HU-14 se restringirá a quienes tuvieron una reserva confirmada. 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.
+12-10-2026: aceptada por el Product Owner. Casos CP-047 y CP-048 aprobados; revisión de código de Luis Méndez en el PR #10.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SC-18: documenta el mapa con MapLibre y OpenFreeMap (DAS 1.23, matriz, casos, defectos 27 a 29, backlog, Guia 2.4 y control)
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -731,7 +731,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="130" customHeight="1">
+    <row r="10" ht="200" customHeight="1">
       <c r="B10" s="9" t="inlineStr">
         <is>
           <t>FS-HU-06</t>
@@ -766,7 +766,8 @@
       <c r="I10" s="9" t="inlineStr">
         <is>
           <t>Mapa/lista integrado por Luis; conserva filtros y página. Pruebas locales aprobadas. Falta clave y validación real Google Maps; revisión y aceptación pendientes. 11-10-2026.
-12-10-2026: los PR #21 y #22 se fusionaron en main (merge 662e79c). Google Maps real comprobado con una Demo Key, sin facturación: marcadores, filtros, Lista/Mapa y paginación. Falta ejecutar CP-078 sobre main y la aceptación del PO.</t>
+12-10-2026: los PR #21 y #22 se fusionaron en main (merge 662e79c). Google Maps real comprobado con una Demo Key, sin facturación: marcadores, filtros, Lista/Mapa y paginación. Falta ejecutar CP-078 sobre main y la aceptación del PO.
+15-10-2026: SC-18 aprobada por el PO. El PR #27 de Nicolás Silva (fusionado) reemplaza Google Maps por MapLibre GL JS con teselas de OpenFreeMap, sin clave ni facturación (DAS 1.23, D31). Falta ejecutar CP-078 sobre main con sesión de usuario, corregir los defectos 27 a 29 y la aceptación del PO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SC-20 y SC-21: reserva con calendario y calendario al publicar horarios
Calendario compartido (CalendarioMes). Reserva: dias con horas, Confirmar en la fila, mensaje obligatorio, solicitud pendiente y archivo .ics. Publicar horario: dia en el calendario, hora de inicio y termino con duracion rapida. CP-088 a CP-093; Guia 2.4, control, matriz, planilla y Product Backlog al 19-10-2026.
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -1020,7 +1020,8 @@
           <t>Agregada el 15-09-2026 (épica E7 Reservas) por decisión del Product Owner y el equipo. Reserva básica sin pagos ni calendarios externos. Replanificada a Sprint 3 (Trello). Sin iniciar; sin responsable ni estimación.
 Avance al 12-10-2026: Arrastre a Sprint 3. Luis implementó API y pantalla; valida futuros, superposición y propiedad. MySQL real aprobado. En revisión, pendiente de fusión y aceptación. 11-10-2026. Corrección del PR #21: comparación en segundos, retiro sin perder historial y prueba MySQL reproducible. En revisión.
 12-10-2026: los PR #21 y #22 se fusionaron en main (merge 662e79c); 55/55 comprobaciones con MySQL real sobre main. Pendiente de aceptación del PO.
-12-10-2026: aceptada por el Product Owner. Casos CP-069 a CP-071 aprobados contra MySQL real; revisión de código de Rodrigo Cárcamo Rojas en los PR #21 y #22.</t>
+12-10-2026: aceptada por el Product Owner. Casos CP-069 a CP-071 aprobados contra MySQL real; revisión de código de Rodrigo Cárcamo Rojas en los PR #21 y #22.
+19-10-2026 (SC-21): «Publicar un horario» usa un calendario en vez del campo de fecha (días pasados deshabilitados, días con horarios marcados), con hora de inicio, hora de término y duración rápida. No cambian los criterios de aceptación, la API ni los datos. CP-092 y CP-093 aprobados.</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1062,8 @@
           <t>Agregada el 15-09-2026 (épica E7 Reservas). Al presionar "Reservar" el usuario escribe un mensaje breve obligatorio para el profesional.
 Avance al 12-10-2026: Luis implementó reserva con mensaje obligatorio, transacción para una activa por bloque, confirmación, cancelación e historial. MySQL real aprobado. En revisión, pendiente de fusión y aceptación. 11-10-2026. Corrección del PR #21: comparación en segundos, retiro sin perder historial y prueba MySQL reproducible. En revisión.
 12-10-2026: el Product Owner definió como máximo una reserva activa (pendiente o confirmada) por usuario con cada profesional; las citas que ya pasaron no cuentan. Implementado en el PR #22 (Luis Méndez, con la corrección de Rodrigo Cárcamo del defecto 26), fusionado el 12-10-2026. Pendiente de aceptación del PO.
-12-10-2026: aceptada por el Product Owner, con observación. Casos CP-072 a CP-075, CP-079 y CP-080 aprobados; revisión de código de Rodrigo Cárcamo Rojas en los PR #21 y #22. Observación: la corrección del defecto 26 (commit 4728310, de Rodrigo Cárcamo Rojas) queda pendiente de revisión por otro integrante (DoD-04).</t>
+12-10-2026: aceptada por el Product Owner, con observación. Casos CP-072 a CP-075, CP-079 y CP-080 aprobados; revisión de código de Rodrigo Cárcamo Rojas en los PR #21 y #22. Observación: la corrección del defecto 26 (commit 4728310, de Rodrigo Cárcamo Rojas) queda pendiente de revisión por otro integrante (DoD-04).
+19-10-2026 (SC-20): se rediseñó la reserva desde la ficha con un calendario del mes, las horas del día con «Confirmar» en la misma fila, el mensaje obligatorio en el paso de confirmar y la pantalla «Solicitud enviada, pendiente de confirmación» con un archivo .ics para el calendario. No cambian los criterios de aceptación, la API ni los datos. CP-088 a CP-091 aprobados.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Defecto 35, SC-22, SC-23 y SC-24: mapa en Chile, detalle en el mapa, buscador general y direccion de atencion
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -688,7 +688,8 @@
         <is>
           <t>06-10-2026 (cierre del Sprint 2): implementada por Luis Méndez en el PR #11 (03-10-2026), en corrección antes de fusionar; pasa al Sprint 3.
 Implementado por Luis (PR #12), con ajustes de Rodri (#13). Pendiente de aceptación del PO. Actualizado 10-10-2026.
-12-10-2026: aceptada por el Product Owner (Rodrigo Cárcamo Rojas).</t>
+12-10-2026: aceptada por el Product Owner (Rodrigo Cárcamo Rojas).
+19-10-2026 (SC-24): la ficha incorpora la dirección de atención (obligatoria salvo que atienda solo online) y solo acepta coordenadas dentro de Chile. Migración aditiva profesionales.direccion. CP-099 y CP-100 aprobados.</t>
         </is>
       </c>
     </row>
@@ -767,7 +768,10 @@
         <is>
           <t>Mapa/lista integrado por Luis; conserva filtros y página. Pruebas locales aprobadas. Falta clave y validación real Google Maps; revisión y aceptación pendientes. 11-10-2026.
 12-10-2026: los PR #21 y #22 se fusionaron en main (merge 662e79c). Google Maps real comprobado con una Demo Key, sin facturación: marcadores, filtros, Lista/Mapa y paginación. Falta ejecutar CP-078 sobre main y la aceptación del PO.
-15-10-2026: SC-18 aprobada por el PO. El PR #27 de Nicolás Silva (fusionado) reemplaza Google Maps por MapLibre GL JS con teselas de OpenFreeMap, sin clave ni facturación (DAS 1.23, D31). Falta ejecutar CP-078 sobre main con sesión de usuario, corregir los defectos 27 a 29 y la aceptación del PO.</t>
+15-10-2026: SC-18 aprobada por el PO. El PR #27 de Nicolás Silva (fusionado) reemplaza Google Maps por MapLibre GL JS con teselas de OpenFreeMap, sin clave ni facturación (DAS 1.23, D31). Falta ejecutar CP-078 sobre main con sesión de usuario, corregir los defectos 27 a 29 y la aceptación del PO.
+19-10-2026: el mapa quedó limitado a Chile; las ubicaciones fuera de Chile no se dibujan ni alejan el encuadre (defecto 35, CP-094). Siguen pendientes CP-078 sobre main y los defectos 27 a 29.
+19-10-2026 (SC-22): la ventana de cada marcador muestra especialidad y modalidad, verificación, lugar de atención y próxima hora disponible, con enlaces a la ficha y a «Cómo llegar»; con el teclado también funciona (defecto 28 corregido). CP-095 y CP-096 aprobados. Siguen pendientes CP-078 y los defectos 27 y 29.
+19-10-2026 (SC-24): la ventana del marcador muestra la dirección que el profesional indica en su ficha (o la de su establecimiento; si atiende solo online, lo dice).</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1335,8 @@
       <c r="I25" s="9" t="inlineStr">
         <is>
           <t>Agregada el 03-10-2026 (épica E1) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Las secciones que aún no existen (centros de salud, gimnasios, farmacias, asistente IA, historial de chats y citas) se muestran como "Próximamente"; la barra de avance del objetivo esperará al gestor de alimentación (FS-HU-09 y FS-HU-10). 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.
-12-10-2026: aceptada por el Product Owner. Casos CP-037 a CP-041 y CP-049 aprobados; revisión de código de Luis Méndez en el PR #10. Los cambios del menú del PR #13 los revisó Luis Méndez al integrarlos en el PR #15.</t>
+12-10-2026: aceptada por el Product Owner. Casos CP-037 a CP-041 y CP-049 aprobados; revisión de código de Luis Méndez en el PR #10. Los cambios del menú del PR #13 los revisó Luis Méndez al integrarlos en el PR #15.
+19-10-2026 (SC-23): el buscador «¿Qué necesitas hoy?» del Inicio sugiere secciones de la aplicación, especialidades y, al final, buscar en profesionales (antes solo buscaba profesionales). Sin cambios en la API. CP-097 y CP-098 aprobados.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FS-HU-07 y SC-25: asistente IA con Groq, DAS 1.25 y documentacion
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -794,7 +794,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Planificada</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
@@ -808,7 +808,11 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>21-10-2026: implementada en la rama feat/asistente-ia (SC-25; DAS 1.25, D33). Pantalla /asistente con historial, chats fijados, sugerencias y aviso de emergencias; API /api/asistente; proveedor Groq (plan gratuito) configurable por .env; límite de 30 mensajes por usuario al día. CP-103 a CP-108 aprobados en modo de prueba. Falta CP-109 con la clave real de Groq, la revisión del PR y la aceptación del Product Owner.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="9" t="inlineStr">
@@ -842,7 +846,11 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="I12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>21-10-2026 (SC-25): usará el mismo proveedor del asistente (Groq) y la conversación de FS-HU-07.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="9" t="inlineStr">

</xml_diff>

<commit_message>
FS-HU-08 y SC-26: recomendacion de profesional y SAMU solo en situaciones criticas (DAS 1.26)
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -811,7 +811,8 @@
       <c r="I11" s="9" t="inlineStr">
         <is>
           <t>21-10-2026: implementada en la rama feat/asistente-ia (SC-25; DAS 1.25, D33). Pantalla /asistente con historial, chats fijados, sugerencias y aviso de emergencias; API /api/asistente; proveedor Groq (plan gratuito) configurable por .env; límite de 30 mensajes por usuario al día. CP-103 a CP-108 aprobados en modo de prueba. Falta CP-109 con la clave real de Groq, la revisión del PR y la aceptación del Product Owner.
-22-10-2026: CP-109 aprobado con Groq real (modelo openai/gpt-oss-120b; el anterior ya no existía, defecto 36). Falta el PR (después del PR #28) y la aceptación del Product Owner.</t>
+22-10-2026: CP-109 aprobado con Groq real (modelo openai/gpt-oss-120b; el anterior ya no existía, defecto 36). Falta el PR (después del PR #28) y la aceptación del Product Owner.
+22-10-2026 (SC-26): el SAMU (131) solo ante situaciones críticas, no en molestias leves ni fijo en el pie del chat (CP-113); escenario 3 agregado en la planilla de historias.</t>
         </is>
       </c>
     </row>
@@ -833,7 +834,7 @@
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Planificada</t>
+          <t>En Proceso</t>
         </is>
       </c>
       <c r="F12" s="9" t="n">
@@ -849,7 +850,8 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>21-10-2026 (SC-25): usará el mismo proveedor del asistente (Groq) y la conversación de FS-HU-07.</t>
+          <t>21-10-2026 (SC-25): usará el mismo proveedor del asistente (Groq) y la conversación de FS-HU-07.
+22-10-2026: implementada en la rama feat/asistente-ia (DAS 1.26, D34). El asistente recomienda una especialidad del catálogo, validada por el backend, con una tarjeta que abre el buscador filtrado; columna mensajes.especialidad (migración aditiva). Cumple los escenarios 1 y 2 de la planilla de historias; se agregó el escenario 3. CP-110 a CP-112 y CP-114 aprobados con Groq real. Falta el PR (después del PR #28) y la aceptación del Product Owner.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Product Backlog: PR 29 y 30 abiertos para FS-HU-06, FS-HU-07 y FS-HU-08
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -773,7 +773,8 @@
 19-10-2026 (SC-22): la ventana de cada marcador muestra especialidad y modalidad, verificación, lugar de atención y próxima hora disponible, con enlaces a la ficha y a «Cómo llegar»; con el teclado también funciona (defecto 28 corregido). CP-095 y CP-096 aprobados. Siguen pendientes CP-078 y los defectos 27 y 29.
 19-10-2026 (SC-24): la ventana del marcador muestra la dirección que el profesional indica en su ficha (o la de su establecimiento; si atiende solo online, lo dice).
 21-10-2026: corregidos los defectos 27 (reintento cuando falla el estilo del mapa) y 29 (controles en español). CP-101 y CP-102 aprobados. Para cerrar la historia falta CP-078 sobre main y la aceptación del Product Owner.
-22-10-2026 (SC-27): la lista y el mapa se ven juntos (en celular, el mapa arriba de la lista); el detalle del marcador elegido pasa de la ventana sobre el marcador a un panel bajo el mapa, «Ver en el mapa» en cada tarjeta, accesos por especialidad, filtros en una barra y opción de ocultar el mapa. Escenarios 1 y 2 de la planilla de historias actualizados y escenario 3 agregado. CP-115 a CP-120 aprobados; defecto 37 corregido. Para cerrar la historia siguen pendientes CP-078 sobre main y la aceptación del Product Owner.</t>
+22-10-2026 (SC-27): la lista y el mapa se ven juntos (en celular, el mapa arriba de la lista); el detalle del marcador elegido pasa de la ventana sobre el marcador a un panel bajo el mapa, «Ver en el mapa» en cada tarjeta, accesos por especialidad, filtros en una barra y opción de ocultar el mapa. Escenarios 1 y 2 de la planilla de historias actualizados y escenario 3 agregado. CP-115 a CP-120 aprobados; defecto 37 corregido. Para cerrar la historia siguen pendientes CP-078 sobre main y la aceptación del Product Owner.
+22-10-2026: PR #30 abierto (rama feat/lista-y-mapa, encadenado sobre el PR #29), con revisión pedida a Nicolás Silva (DoD-04). Se fusiona después de los PR #28 y #29.</t>
         </is>
       </c>
     </row>
@@ -813,7 +814,8 @@
         <is>
           <t>21-10-2026: implementada en la rama feat/asistente-ia (SC-25; DAS 1.25, D33). Pantalla /asistente con historial, chats fijados, sugerencias y aviso de emergencias; API /api/asistente; proveedor Groq (plan gratuito) configurable por .env; límite de 30 mensajes por usuario al día. CP-103 a CP-108 aprobados en modo de prueba. Falta CP-109 con la clave real de Groq, la revisión del PR y la aceptación del Product Owner.
 22-10-2026: CP-109 aprobado con Groq real (modelo openai/gpt-oss-120b; el anterior ya no existía, defecto 36). Falta el PR (después del PR #28) y la aceptación del Product Owner.
-22-10-2026 (SC-26): el SAMU (131) solo ante situaciones críticas, no en molestias leves ni fijo en el pie del chat (CP-113); escenario 3 agregado en la planilla de historias.</t>
+22-10-2026 (SC-26): el SAMU (131) solo ante situaciones críticas, no en molestias leves ni fijo en el pie del chat (CP-113); escenario 3 agregado en la planilla de historias.
+22-10-2026: PR #29 abierto (rama feat/asistente-ia, encadenado sobre el PR #28), con revisión pedida a Luis Méndez (DoD-04). Se fusiona después del PR #28.</t>
         </is>
       </c>
     </row>
@@ -852,7 +854,8 @@
       <c r="I12" s="9" t="inlineStr">
         <is>
           <t>21-10-2026 (SC-25): usará el mismo proveedor del asistente (Groq) y la conversación de FS-HU-07.
-22-10-2026: implementada en la rama feat/asistente-ia (DAS 1.26, D34). El asistente recomienda una especialidad del catálogo, validada por el backend, con una tarjeta que abre el buscador filtrado; columna mensajes.especialidad (migración aditiva). Cumple los escenarios 1 y 2 de la planilla de historias; se agregó el escenario 3. CP-110 a CP-112 y CP-114 aprobados con Groq real. Falta el PR (después del PR #28) y la aceptación del Product Owner.</t>
+22-10-2026: implementada en la rama feat/asistente-ia (DAS 1.26, D34). El asistente recomienda una especialidad del catálogo, validada por el backend, con una tarjeta que abre el buscador filtrado; columna mensajes.especialidad (migración aditiva). Cumple los escenarios 1 y 2 de la planilla de historias; se agregó el escenario 3. CP-110 a CP-112 y CP-114 aprobados con Groq real. Falta el PR (después del PR #28) y la aceptación del Product Owner.
+22-10-2026: PR #29 abierto (rama feat/asistente-ia, encadenado sobre el PR #28), con revisión pedida a Luis Méndez (DoD-04). Se fusiona después del PR #28.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Defectos 38 y 39: CP-121 y CP-122, Product Backlog y control del proyecto
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -815,7 +815,9 @@
           <t>21-10-2026: implementada en la rama feat/asistente-ia (SC-25; DAS 1.25, D33). Pantalla /asistente con historial, chats fijados, sugerencias y aviso de emergencias; API /api/asistente; proveedor Groq (plan gratuito) configurable por .env; límite de 30 mensajes por usuario al día. CP-103 a CP-108 aprobados en modo de prueba. Falta CP-109 con la clave real de Groq, la revisión del PR y la aceptación del Product Owner.
 22-10-2026: CP-109 aprobado con Groq real (modelo openai/gpt-oss-120b; el anterior ya no existía, defecto 36). Falta el PR (después del PR #28) y la aceptación del Product Owner.
 22-10-2026 (SC-26): el SAMU (131) solo ante situaciones críticas, no en molestias leves ni fijo en el pie del chat (CP-113); escenario 3 agregado en la planilla de historias.
-22-10-2026: PR #29 abierto (rama feat/asistente-ia, encadenado sobre el PR #28), con revisión pedida a Luis Méndez (DoD-04). Se fusiona después del PR #28.</t>
+22-10-2026: PR #29 abierto (rama feat/asistente-ia, encadenado sobre el PR #28), con revisión pedida a Luis Méndez (DoD-04). Se fusiona después del PR #28.
+22-10-2026 (defecto 38): la red de seguridad no reconocía «me quiero matar», «quiero morir» y frases parecidas; corregido en el PR #29 antes de su revisión (CP-121).
+23-10-2026 (defecto 39): Nicolás Silva pidió cambios en el PR #29 porque el límite diario se podía superar con mensajes simultáneos (29 de 30 usados y tres a la vez llegaban a 32). Corregido en el PR #29: el cupo se reserva de forma atómica antes de llamar al proveedor y se devuelve si falla (CP-122). Falta su nueva revisión.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CP-078 aprobado sobre main con el mapa real (FS-HU-06)
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -774,7 +774,9 @@
 19-10-2026 (SC-24): la ventana del marcador muestra la dirección que el profesional indica en su ficha (o la de su establecimiento; si atiende solo online, lo dice).
 21-10-2026: corregidos los defectos 27 (reintento cuando falla el estilo del mapa) y 29 (controles en español). CP-101 y CP-102 aprobados. Para cerrar la historia falta CP-078 sobre main y la aceptación del Product Owner.
 22-10-2026 (SC-27): la lista y el mapa se ven juntos (en celular, el mapa arriba de la lista); el detalle del marcador elegido pasa de la ventana sobre el marcador a un panel bajo el mapa, «Ver en el mapa» en cada tarjeta, accesos por especialidad, filtros en una barra y opción de ocultar el mapa. Escenarios 1 y 2 de la planilla de historias actualizados y escenario 3 agregado. CP-115 a CP-120 aprobados; defecto 37 corregido. Para cerrar la historia siguen pendientes CP-078 sobre main y la aceptación del Product Owner.
-22-10-2026: PR #30 abierto (rama feat/lista-y-mapa, encadenado sobre el PR #29), con revisión pedida a Nicolás Silva (DoD-04). Se fusiona después de los PR #28 y #29.</t>
+22-10-2026: PR #30 abierto (rama feat/lista-y-mapa, encadenado sobre el PR #29), con revisión pedida a Nicolás Silva (DoD-04). Se fusiona después de los PR #28 y #29.
+23-10-2026: Luis Méndez revisó y aprobó el PR #30, que se fusionó en main después del PR #29.
+24-10-2026: CP-078 aprobado sobre main con el mapa real (MapLibre GL JS y OpenFreeMap): un marcador por cada resultado de la página, con filtros, páginas y mapa oculto, y cada marcador ofrece su ficha. Solo falta la aceptación del Product Owner.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SC-29: rediseño de portada e Inicio, defectos 40 y 41 y CP-126 a CP-130
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -1317,7 +1317,8 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>Agregada el 23-09-2026 (épica E1). La portada la construyó Nicolás Silva (PR #2, 22-09-2026); el 23-09-2026 el Product Owner definió que es solo para quien no ha iniciado sesión: con la sesión iniciada se va directo al perfil y al cerrar sesión se vuelve a la portada. 23-09-2026: implementada y probada (CP-020 a CP-023); falta completar la DoD (revisión de código). 03-10-2026: con la sesión iniciada la raíz lleva al Inicio (/inicio, FS-HU-21) en vez del perfil, y la portada se rediseñó con la propuesta "Tu salud y bienestar, en un solo lugar" y lo que ofrece FitSearch (CP-036 y CP-037). 03-10-2026: aceptada por el Product Owner, con la revisión de código aprobada por Luis Méndez en el PR #9. El código de la portada entró por el PR #2, que se fusionó sin revisión; la revisión se hizo después en el PR #9.</t>
+          <t>Agregada el 23-09-2026 (épica E1). La portada la construyó Nicolás Silva (PR #2, 22-09-2026); el 23-09-2026 el Product Owner definió que es solo para quien no ha iniciado sesión: con la sesión iniciada se va directo al perfil y al cerrar sesión se vuelve a la portada. 23-09-2026: implementada y probada (CP-020 a CP-023); falta completar la DoD (revisión de código). 03-10-2026: con la sesión iniciada la raíz lleva al Inicio (/inicio, FS-HU-21) en vez del perfil, y la portada se rediseñó con la propuesta "Tu salud y bienestar, en un solo lugar" y lo que ofrece FitSearch (CP-036 y CP-037). 03-10-2026: aceptada por el Product Owner, con la revisión de código aprobada por Luis Méndez en el PR #9. El código de la portada entró por el PR #2, que se fusionó sin revisión; la revisión se hizo después en el PR #9.
+26-10-2026 (SC-29): rediseño de la portada propuesto por Luis Méndez (PR #33) y aceptado por el Product Owner: escena del centro de bienestar con puertas que se abren al bajar (bienvenida, especialidades y asistente IA), estilo translúcido y buscador por especialidad y comuna que conserva los filtros al iniciar sesión. Defectos 40 y 41 corregidos en la revisión. CP-126 a CP-129 aprobados. La historia sigue Hecho.</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1358,8 @@
         <is>
           <t>Agregada el 03-10-2026 (épica E1) por decisión del Product Owner a partir del mockup del Inicio. Implementada y probada el 03-10-2026, antes del inicio del Sprint 3 (casos CP-036 a CP-049); falta completar la DoD (revisión de código y PR). La estimación es una propuesta: el equipo la confirma en la planificación del Sprint 3. Las secciones que aún no existen (centros de salud, gimnasios, farmacias, asistente IA, historial de chats y citas) se muestran como "Próximamente"; la barra de avance del objetivo esperará al gestor de alimentación (FS-HU-09 y FS-HU-10). 03-10-2026: revisión de código aprobada por Luis Méndez y fusionada en main (PR #10); falta la aceptación del Product Owner.
 12-10-2026: aceptada por el Product Owner. Casos CP-037 a CP-041 y CP-049 aprobados; revisión de código de Luis Méndez en el PR #10. Los cambios del menú del PR #13 los revisó Luis Méndez al integrarlos en el PR #15.
-19-10-2026 (SC-23): el buscador «¿Qué necesitas hoy?» del Inicio sugiere secciones de la aplicación, especialidades y, al final, buscar en profesionales (antes solo buscaba profesionales). Sin cambios en la API. CP-097 y CP-098 aprobados.</t>
+19-10-2026 (SC-23): el buscador «¿Qué necesitas hoy?» del Inicio sugiere secciones de la aplicación, especialidades y, al final, buscar en profesionales (antes solo buscaba profesionales). Sin cambios en la API. CP-097 y CP-098 aprobados.
+26-10-2026 (SC-29): rediseño del Inicio en el mismo PR #33 (saludo, fotografía, tarjetas por especialidad y asistente destacado), con los mismos datos reales. CP-130 aprobado. La historia sigue Hecho.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aceptacion del PO de FS-HU-06, FS-HU-07 y FS-HU-08
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/PMOInformatica_Plantilla_de_Product_Backlog.xlsx
@@ -690,7 +690,8 @@
 Implementado por Luis (PR #12), con ajustes de Rodri (#13). Pendiente de aceptación del PO. Actualizado 10-10-2026.
 12-10-2026: aceptada por el Product Owner (Rodrigo Cárcamo Rojas).
 19-10-2026 (SC-24): la ficha incorpora la dirección de atención (obligatoria salvo que atienda solo online) y solo acepta coordenadas dentro de Chile. Migración aditiva profesionales.direccion. CP-099 y CP-100 aprobados.
-24-10-2026 (SC-28): el profesional ya no escribe coordenadas: indica su comuna y su dirección, la API las ubica con Nominatim (OpenStreetMap) y el formulario muestra un mapa con el marcador, que puede ajustar arrastrándolo, con un clic o con las flechas. CP-123 a CP-125 aprobados. Rama feat/ubicacion-por-direccion, pendiente de PR y revisión.</t>
+24-10-2026 (SC-28): el profesional ya no escribe coordenadas: indica su comuna y su dirección, la API las ubica con Nominatim (OpenStreetMap) y el formulario muestra un mapa con el marcador, que puede ajustar arrastrándolo, con un clic o con las flechas. CP-123 a CP-125 aprobados. Rama feat/ubicacion-por-direccion, pendiente de PR y revisión.
+25-10-2026: la SC-28 entró a main con el PR #32, fusionado sin revisión de otro integrante; queda pendiente esa revisión (DoD-04).</t>
         </is>
       </c>
     </row>
@@ -751,7 +752,7 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F10" s="9" t="n">
@@ -777,7 +778,8 @@
 22-10-2026 (SC-27): la lista y el mapa se ven juntos (en celular, el mapa arriba de la lista); el detalle del marcador elegido pasa de la ventana sobre el marcador a un panel bajo el mapa, «Ver en el mapa» en cada tarjeta, accesos por especialidad, filtros en una barra y opción de ocultar el mapa. Escenarios 1 y 2 de la planilla de historias actualizados y escenario 3 agregado. CP-115 a CP-120 aprobados; defecto 37 corregido. Para cerrar la historia siguen pendientes CP-078 sobre main y la aceptación del Product Owner.
 22-10-2026: PR #30 abierto (rama feat/lista-y-mapa, encadenado sobre el PR #29), con revisión pedida a Nicolás Silva (DoD-04). Se fusiona después de los PR #28 y #29.
 23-10-2026: Luis Méndez revisó y aprobó el PR #30, que se fusionó en main después del PR #29.
-24-10-2026: CP-078 aprobado sobre main con el mapa real (MapLibre GL JS y OpenFreeMap): un marcador por cada resultado de la página, con filtros, páginas y mapa oculto, y cada marcador ofrece su ficha. Solo falta la aceptación del Product Owner.</t>
+24-10-2026: CP-078 aprobado sobre main con el mapa real (MapLibre GL JS y OpenFreeMap): un marcador por cada resultado de la página, con filtros, páginas y mapa oculto, y cada marcador ofrece su ficha. Solo falta la aceptación del Product Owner.
+26-10-2026: aceptada por el Product Owner (Sprint 4). PR #21, #22, #27, #28 y #30 fusionados en main; CP-076 a CP-078, CP-094 a CP-096, CP-101, CP-102 y CP-115 a CP-120 aprobados.</t>
         </is>
       </c>
     </row>
@@ -799,7 +801,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
@@ -820,7 +822,8 @@
 22-10-2026 (SC-26): el SAMU (131) solo ante situaciones críticas, no en molestias leves ni fijo en el pie del chat (CP-113); escenario 3 agregado en la planilla de historias.
 22-10-2026: PR #29 abierto (rama feat/asistente-ia, encadenado sobre el PR #28), con revisión pedida a Luis Méndez (DoD-04). Se fusiona después del PR #28.
 22-10-2026 (defecto 38): la red de seguridad no reconocía «me quiero matar», «quiero morir» y frases parecidas; corregido en el PR #29 antes de su revisión (CP-121).
-23-10-2026 (defecto 39): Luis Méndez pidió cambios en el PR #29 porque el límite diario se podía superar con mensajes simultáneos (29 de 30 usados y tres a la vez llegaban a 32). Corregido en el PR #29: el cupo se reserva de forma atómica antes de llamar al proveedor y se devuelve si falla (CP-122). Luis lo aprobó tras agregar un ajuste (el reinicio de día solo avanza) y 23 comprobaciones con MySQL real; PR #29 fusionado en main el 23-10-2026. Falta la aceptación del Product Owner.</t>
+23-10-2026 (defecto 39): Luis Méndez pidió cambios en el PR #29 porque el límite diario se podía superar con mensajes simultáneos (29 de 30 usados y tres a la vez llegaban a 32). Corregido en el PR #29: el cupo se reserva de forma atómica antes de llamar al proveedor y se devuelve si falla (CP-122). Luis lo aprobó tras agregar un ajuste (el reinicio de día solo avanza) y 23 comprobaciones con MySQL real; PR #29 fusionado en main el 23-10-2026. Falta la aceptación del Product Owner.
+26-10-2026: aceptada por el Product Owner, junto con FS-HU-08. PR #29 fusionado en main; CP-103 a CP-109, CP-113, CP-121 y CP-122 aprobados.</t>
         </is>
       </c>
     </row>
@@ -842,7 +845,7 @@
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>En Proceso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F12" s="9" t="n">
@@ -860,7 +863,9 @@
         <is>
           <t>21-10-2026 (SC-25): usará el mismo proveedor del asistente (Groq) y la conversación de FS-HU-07.
 22-10-2026: implementada en la rama feat/asistente-ia (DAS 1.26, D34). El asistente recomienda una especialidad del catálogo, validada por el backend, con una tarjeta que abre el buscador filtrado; columna mensajes.especialidad (migración aditiva). Cumple los escenarios 1 y 2 de la planilla de historias; se agregó el escenario 3. CP-110 a CP-112 y CP-114 aprobados con Groq real. Falta el PR (después del PR #28) y la aceptación del Product Owner.
-22-10-2026: PR #29 abierto (rama feat/asistente-ia, encadenado sobre el PR #28), con revisión pedida a Luis Méndez (DoD-04). Se fusiona después del PR #28.</t>
+22-10-2026: PR #29 abierto (rama feat/asistente-ia, encadenado sobre el PR #28), con revisión pedida a Luis Méndez (DoD-04). Se fusiona después del PR #28.
+23-10-2026: PR #29 aprobado por Luis Méndez y fusionado en main.
+26-10-2026: aceptada por el Product Owner, junto con FS-HU-07. CP-110 a CP-112 y CP-114 aprobados.</t>
         </is>
       </c>
     </row>

</xml_diff>